<commit_message>
changes done on registration page
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c2cdd42149d18ae4/Desktop/Jan 2025 Batch Selenium Java/BreakOut_GitHubJenkinsFreamwork/SeleniumFrameworkJanBatch2025/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_C23BD98C8EAF39736A2ED3D95BBEB7055CA6C671" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEA3ABCC-089F-4E88-9616-F7786887651B}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_C23BD98C8EAF39736A2ED3D95BBEB7055CA6C671" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C3718F0-22B7-47B3-A2DE-1C41AADBE762}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,9 +61,6 @@
     <t>testAnotherUser@gmail.com</t>
   </si>
   <si>
-    <t>pass1</t>
-  </si>
-  <si>
     <t>Female</t>
   </si>
   <si>
@@ -74,6 +71,9 @@
   </si>
   <si>
     <t>C#</t>
+  </si>
+  <si>
+    <t>pass145</t>
   </si>
 </sst>
 </file>
@@ -307,7 +307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200B2865-0703-462C-AF0C-33C94DEFBE3A}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.26953125" bestFit="1" customWidth="1"/>
@@ -346,173 +346,20 @@
         <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>